<commit_message>
Show the 462 selection and 5 µm copy status on the progress overview.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/group_analysis/evolution_20261008/overview_legacy_plot_20261012/data_progress_table.xlsx
+++ b/group_analysis/evolution_20261008/overview_legacy_plot_20261012/data_progress_table.xlsx
@@ -12,7 +12,7 @@
     <sheet name="totals" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'progress'!$A$1:$AK$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'progress'!$A$1:$AM$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK11"/>
+  <dimension ref="A1:AM11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -623,15 +623,25 @@
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
+          <t>selected_n</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
           <t>insula_8_cohort</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>cohort_bar_n</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>five_um_folder</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>progress_details_source</t>
         </is>
@@ -640,7 +650,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -792,17 +802,27 @@
           <t>260</t>
         </is>
       </c>
-      <c r="AI2" s="3" t="inlineStr">
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="AJ2" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>212</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>251637-CH1_resample</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -811,7 +831,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -877,7 +897,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>No,to copy</t>
+          <t>no local copy</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -959,17 +979,23 @@
         </is>
       </c>
       <c r="AH3" t="inlineStr"/>
-      <c r="AI3" s="3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="AJ3" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr">
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -978,7 +1004,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1126,17 +1152,27 @@
         </is>
       </c>
       <c r="AH4" t="inlineStr"/>
-      <c r="AI4" s="3" t="inlineStr">
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="AJ4" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>252385-CH1_resample</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -1145,7 +1181,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1211,7 +1247,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>No,to copy</t>
+          <t>no local copy</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -1289,17 +1325,23 @@
         </is>
       </c>
       <c r="AH5" t="inlineStr"/>
-      <c r="AI5" s="3" t="inlineStr">
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="AJ5" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AK5" t="inlineStr">
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -1308,7 +1350,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1374,7 +1416,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>No,to copy</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -1456,17 +1498,27 @@
         </is>
       </c>
       <c r="AH6" t="inlineStr"/>
-      <c r="AI6" s="3" t="inlineStr">
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="AJ6" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ6" t="inlineStr">
+      <c r="AK6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="AK6" t="inlineStr">
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>252384_CH1_resample</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -1475,7 +1527,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1541,7 +1593,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>No,to copy</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R7" t="n">
@@ -1623,17 +1675,27 @@
         </is>
       </c>
       <c r="AH7" t="inlineStr"/>
-      <c r="AI7" s="3" t="inlineStr">
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="AJ7" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ7" t="inlineStr">
+      <c r="AK7" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="AK7" t="inlineStr">
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>252527_CH1_resample</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -1642,7 +1704,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1708,7 +1770,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>No,to copy</t>
+          <t>no local copy</t>
         </is>
       </c>
       <c r="R8" t="n">
@@ -1786,17 +1848,23 @@
         </is>
       </c>
       <c r="AH8" t="inlineStr"/>
-      <c r="AI8" s="3" t="inlineStr">
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="AJ8" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ8" t="inlineStr">
+      <c r="AK8" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="AK8" t="inlineStr">
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -1805,7 +1873,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1871,7 +1939,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R9" t="n">
@@ -1949,17 +2017,27 @@
         </is>
       </c>
       <c r="AH9" t="inlineStr"/>
-      <c r="AI9" s="3" t="inlineStr">
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="AJ9" s="3" t="inlineStr">
         <is>
           <t>DEB lab</t>
         </is>
       </c>
-      <c r="AJ9" t="inlineStr">
+      <c r="AK9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AK9" t="inlineStr">
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>252714-CH1_resample</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -1994,7 +2072,11 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>no local copy</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
@@ -2060,13 +2142,15 @@
         </is>
       </c>
       <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr">
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr">
         <is>
           <t>Other lab</t>
         </is>
       </c>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr">
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
@@ -2075,7 +2159,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2090,7 +2174,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8 plan + 1 outside</t>
+          <t>Table total, 9 animals</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2147,7 +2231,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>5/9</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -2162,7 +2246,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>ION 1498/2429; insula 301/2400; combined 306; 5µm 2/8; 1 animals outside the DEB lab eight remain after dropping rows with no insula neuron</t>
+          <t>Selected is the 462-neuron ledger. 747 is not in that ledger and is not added to Selected. ARM and spatial is the intersection already inside ARM insula and is not added again. DEB lab summary is separate: 8 monkeys, screened 1498, ARM insula 301, plan target 2400.</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -2212,47 +2296,53 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
+          <t>1732</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr">
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>462</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Table total</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AF11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AJ11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AK11" t="inlineStr">
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr">
         <is>
           <t>tsv_fallback:progress_details_BB08J2.tsv</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK11"/>
+  <autoFilter ref="A1:AM11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2624,7 +2714,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-12 14:30 China Standard Time</t>
+          <t>2026-10-12 17:58 China Standard Time</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2726,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20261012_1430</t>
+          <t>20261012_1758</t>
         </is>
       </c>
     </row>

</xml_diff>